<commit_message>
building reconcile pipeline & reset main kg
</commit_message>
<xml_diff>
--- a/reconcile/storage/output/factory-technological.xlsx
+++ b/reconcile/storage/output/factory-technological.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E127"/>
+  <dimension ref="A1:H127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -449,6 +449,21 @@
           <t>product_id</t>
         </is>
       </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>factory_name</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>factory_city</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>factory_country</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
@@ -474,6 +489,17 @@
           <t>67f52a45981040986eab706f_product_s500e</t>
         </is>
       </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Thailand Factory</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Thailand</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
@@ -499,6 +525,17 @@
           <t>67f52a45981040986eab706f_product_c350e</t>
         </is>
       </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Thailand Factory</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Thailand</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
@@ -524,6 +561,21 @@
           <t>67f52a48981040986eab707b_product_battery</t>
         </is>
       </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Saxony Factory</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Saxony</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
@@ -549,6 +601,17 @@
           <t>67f52a4a981040986eab7083_product_fuel_cell_two_seater_rasa</t>
         </is>
       </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Welsh Production Plant</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Wales</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
@@ -574,6 +637,21 @@
           <t>67f52a4e981040986eab7091_product_ioniq_electric</t>
         </is>
       </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Wuhu</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Wuhu</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
@@ -599,6 +677,21 @@
           <t>67f52a51981040986eab709d_product_li_ion_batteries</t>
         </is>
       </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>BMZ Karlstein-Großwelzheim</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Karlstein-Großwelzheim</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
@@ -624,6 +717,21 @@
           <t>67f52a51981040986eab709f_product_electric_buses</t>
         </is>
       </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Qingdao Facility</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Qingdao</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
@@ -649,6 +757,21 @@
           <t>67f52a51981040986eab709f_product_electric_buses</t>
         </is>
       </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Qingdao Facility</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Qingdao</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
@@ -674,6 +797,21 @@
           <t>67f52a52981040986eab70a3_product_streetscooter_van</t>
         </is>
       </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Aachen</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Aachen</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
@@ -699,6 +837,21 @@
           <t>67f52a52981040986eab70a3_product_compact_electric_cars</t>
         </is>
       </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Zhejiang</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Zhejiang</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
@@ -724,6 +877,21 @@
           <t>67f52a53981040986eab70a6_product_electric_bus</t>
         </is>
       </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Komárom</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Komárom</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Hungary</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
@@ -749,6 +917,21 @@
           <t>67f52a54981040986eab70a8_product_batteries</t>
         </is>
       </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Quinghai Battery Factory</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Quinghai</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
@@ -774,6 +957,13 @@
           <t>67f52a56981040986eab70b2_product_powerwall</t>
         </is>
       </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Gigafactory</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
@@ -799,6 +989,13 @@
           <t>67f52a56981040986eab70b2_product_powerwall</t>
         </is>
       </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Gigafactory</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
@@ -824,6 +1021,21 @@
           <t>67f52a57981040986eab70b4_product_battery_packs</t>
         </is>
       </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>3K One</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>northern Austria</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
@@ -849,6 +1061,21 @@
           <t>67f52a57981040986eab70b5_product_lithium_carbonate</t>
         </is>
       </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Qinghai Lithium Carbonate Plant</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Qinghai</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
@@ -874,6 +1101,17 @@
           <t>67f52a58981040986eab70bb_product_ev_battery</t>
         </is>
       </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Poland EV Battery</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Poland</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
@@ -899,6 +1137,17 @@
           <t>67f52a59981040986eab70be_electric_bus</t>
         </is>
       </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>assembly plant</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Thailand</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
@@ -924,6 +1173,21 @@
           <t>67f52a59981040986eab70bf_product_electric_hybrid_cars</t>
         </is>
       </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Tianjin EV Component Factory</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Tianjin</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
@@ -949,6 +1213,21 @@
           <t>67f52a5b981040986eab70c6_product_electric_buses</t>
         </is>
       </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Taiyuan Plant</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Taiyuan</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
@@ -974,6 +1253,21 @@
           <t>67f52a5b981040986eab70c6_product_special_purpose_vehicles</t>
         </is>
       </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Taiyuan Plant</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Taiyuan</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
@@ -999,6 +1293,21 @@
           <t>67f52a5f981040986eab70d4_product_trumpchi_cars_ev</t>
         </is>
       </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Xinjiang Factory</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Xinjiang</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
@@ -1024,6 +1333,21 @@
           <t>67f52a5f981040986eab70d4_product_trumpchi_cars_ev</t>
         </is>
       </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Xinjiang Factory</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Xinjiang</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
@@ -1049,6 +1373,21 @@
           <t>67f52a60981040986eab70d9_product_q6_etron</t>
         </is>
       </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Brussel Facility</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Brussel</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Belgium</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
@@ -1074,6 +1413,21 @@
           <t>67f52a62981040986eab70e1_product_high_performance_motors_and_components</t>
         </is>
       </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Nanjing Facility</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Nanjing</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
@@ -1099,6 +1453,21 @@
           <t>67f52a62981040986eab70e1_product_qiantu_k50</t>
         </is>
       </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Suzhou Factory</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Suzhou</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
@@ -1124,6 +1493,13 @@
           <t>67f52a63981040986eab70e5_product_battery_cells</t>
         </is>
       </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Gigafactory</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
@@ -1149,6 +1525,21 @@
           <t>67f52a63981040986eab70e7_product_nikola_one</t>
         </is>
       </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Guizhou Factory</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Guizhou</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
@@ -1174,6 +1565,13 @@
           <t>67f52a65981040986eab70ee_product_lithium</t>
         </is>
       </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>lithium production plant</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
@@ -1199,6 +1597,17 @@
           <t>67f52a66981040986eab70f0_product_lithium_hydroxide</t>
         </is>
       </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Australia EV battery plant</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
@@ -1224,6 +1633,21 @@
           <t>67f52a67981040986eab70f4_product_battery_packs</t>
         </is>
       </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Budapest Battery Plant</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Budapest</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Hungary</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
@@ -1249,6 +1673,13 @@
           <t>67f52a68981040986eab70f8_product_powerpack_system</t>
         </is>
       </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Southern California Edison facility</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
@@ -1274,6 +1705,21 @@
           <t>67f52a68981040986eab70f9_product_ev</t>
         </is>
       </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Fremont</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Fremont</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
@@ -1299,6 +1745,17 @@
           <t>67f52a68981040986eab70fb_product_electric_cars</t>
         </is>
       </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Future Mobility facility</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
@@ -1324,6 +1781,17 @@
           <t>67f52a68981040986eab70fb_product_batteries</t>
         </is>
       </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Future Mobility facility</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr"/>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
@@ -1349,6 +1817,21 @@
           <t>67f52a6b981040986eab7105_product_ev_batteries</t>
         </is>
       </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Seosan Plant</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Seosan</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>South Korea</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
@@ -1374,6 +1857,21 @@
           <t>67f52a6c981040986eab7108_product_electric_buses</t>
         </is>
       </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Hebei Facility</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Hebei</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
@@ -1399,6 +1897,17 @@
           <t>67f52a6e981040986eab7111_product_electrolytes</t>
         </is>
       </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>electrolyte production facility</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr"/>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
@@ -1424,6 +1933,21 @@
           <t>67f52a6e981040986eab7112_product_electric_buses</t>
         </is>
       </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Xi'an Plant</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Xi'an</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
@@ -1449,6 +1973,21 @@
           <t>67f52a71981040986eab711c_product_ev_batteries</t>
         </is>
       </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Seosan Plant</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Seosan</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>South Korea</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
@@ -1474,6 +2013,21 @@
           <t>67f52a72981040986eab7122_product_electric_buses</t>
         </is>
       </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>BYD Electric Bus &amp; Truck Hungary</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Komárom</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Hungary</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
@@ -1499,6 +2053,21 @@
           <t>67f52a72981040986eab7122_product_forklifts</t>
         </is>
       </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>BYD Electric Bus &amp; Truck Hungary</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Komárom</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Hungary</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
@@ -1524,6 +2093,21 @@
           <t>67f52a72981040986eab7123_electric_buses</t>
         </is>
       </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Lancaster Plant</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Lancaster</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="n">
@@ -1549,6 +2133,21 @@
           <t>67f52a73981040986eab7125_product_ev_batteries</t>
         </is>
       </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Kobierzyce Facility</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Kobierzyce</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Poland</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="n">
@@ -1574,6 +2173,21 @@
           <t>67f52a73981040986eab7126_product_electric_cars</t>
         </is>
       </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Tongling Facility</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Tongling</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="n">
@@ -1599,6 +2213,17 @@
           <t>67f52a78981040986eab713a_product_electric_buses</t>
         </is>
       </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Ecuador Facility</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr"/>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="n">
@@ -1624,6 +2249,21 @@
           <t>67f52a7a981040986eab7140_product_lithium_batteries</t>
         </is>
       </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Fujian Assembly Facility</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Fujian</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="n">
@@ -1649,6 +2289,21 @@
           <t>67f52a7a981040986eab7140_product_lithium_batteries</t>
         </is>
       </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Hubei Plant</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Hubei</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="n">
@@ -1674,6 +2329,21 @@
           <t>67f52a7a981040986eab7142_product_ev_battery</t>
         </is>
       </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Vernon Factory</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Vernon</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="1" t="n">
@@ -1699,6 +2369,21 @@
           <t>67f52a7a981040986eab7142_product_ev_battery</t>
         </is>
       </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Vernon Factory</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Vernon</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="1" t="n">
@@ -1724,6 +2409,21 @@
           <t>67f52a7a981040986eab7142_product_ev_battery</t>
         </is>
       </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Vernon Factory</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Vernon</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="1" t="n">
@@ -1749,6 +2449,21 @@
           <t>67f52a7b981040986eab7147_product_electric_suv</t>
         </is>
       </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Nanjing Factory</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Nanjing</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="1" t="n">
@@ -1774,6 +2489,21 @@
           <t>67f52a7c981040986eab7149_product_electric_buses</t>
         </is>
       </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Allonne Plant</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Allonne</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="1" t="n">
@@ -1799,6 +2529,21 @@
           <t>67f52a7c981040986eab714a_product_electric_cabs</t>
         </is>
       </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Ansty Plant</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Ansty</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="1" t="n">
@@ -1824,6 +2569,21 @@
           <t>67f52a7c981040986eab714a_product_electric_buses</t>
         </is>
       </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Bursa Factory</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Bursa</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Turkey</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="1" t="n">
@@ -1849,6 +2609,17 @@
           <t>67f52a7d981040986eab714f_product_lithium_carbonate</t>
         </is>
       </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>lithium factory</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr"/>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="1" t="n">
@@ -1874,6 +2645,17 @@
           <t>67f52a7d981040986eab714f_product_lithium_carbonate</t>
         </is>
       </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>lithium factory</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr"/>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="1" t="n">
@@ -1899,6 +2681,17 @@
           <t>67f52a7e981040986eab7150_product_electric_cars</t>
         </is>
       </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr"/>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="1" t="n">
@@ -1924,6 +2717,17 @@
           <t>67f52a7e981040986eab7150_product_plug_in_hybrid_vehicles</t>
         </is>
       </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr"/>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="1" t="n">
@@ -1949,6 +2753,21 @@
           <t>67f52a7f981040986eab7154_product_battery</t>
         </is>
       </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Gigafactory</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>Reno</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="1" t="n">
@@ -1974,6 +2793,21 @@
           <t>67f52a7f981040986eab7156_product_li_ion_batteries</t>
         </is>
       </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Ningbo Plant</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>Ningbo</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="1" t="n">
@@ -1999,6 +2833,21 @@
           <t>67f52a82981040986eab7161_product_ev</t>
         </is>
       </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Tianjin Factory</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>Tianjin</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="1" t="n">
@@ -2024,6 +2873,21 @@
           <t>67f52a82981040986eab7163_product_electric_buses</t>
         </is>
       </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>Komárom Plant</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>Komárom</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>Hungary</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="1" t="n">
@@ -2049,6 +2913,17 @@
           <t>67f52a82981040986eab7163_product_electric_buses</t>
         </is>
       </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>France Plant</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr"/>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="1" t="n">
@@ -2074,6 +2949,21 @@
           <t>67f52a83981040986eab7166_product_ultracapacitor_cells</t>
         </is>
       </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>Saxonia Factory</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>Saxonia</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="1" t="n">
@@ -2099,6 +2989,21 @@
           <t>67f52a84981040986eab7168_product_id_concept</t>
         </is>
       </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>Zwickau</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>Zwickau</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="1" t="n">
@@ -2124,6 +3029,21 @@
           <t>67f52a84981040986eab7168_product_ev_buses</t>
         </is>
       </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>Yinchuan</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>Yinchuan</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="1" t="n">
@@ -2149,6 +3069,21 @@
           <t>67f52a84981040986eab716b_product_pi_1</t>
         </is>
       </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>Fujian Production Facility</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>Fujian Province</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="1" t="n">
@@ -2174,6 +3109,21 @@
           <t>67f52a84981040986eab716b_product_pi_3</t>
         </is>
       </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>Fujian Production Facility</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>Fujian Province</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="1" t="n">
@@ -2199,6 +3149,21 @@
           <t>67f52a85981040986eab716d_product_nano_batteries</t>
         </is>
       </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>Ostrava Plant</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>Ostrava</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>Czech Republic</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="1" t="n">
@@ -2224,6 +3189,21 @@
           <t>67f52a85981040986eab716f_product_fuel_cell_truck</t>
         </is>
       </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>Tennessee</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>Tennessee</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="1" t="n">
@@ -2249,6 +3229,21 @@
           <t>67f52a87981040986eab7177_product_battery_cells</t>
         </is>
       </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>Nanjing Factory</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>Nanjing</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="1" t="n">
@@ -2274,6 +3269,17 @@
           <t>67f52a88981040986eab7178_product_electric_drive_systems</t>
         </is>
       </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>Arizona Plant</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr"/>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="1" t="n">
@@ -2299,6 +3305,17 @@
           <t>67f52a88981040986eab7178_product_electric_drive_systems</t>
         </is>
       </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>Arizona Plant</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr"/>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="1" t="n">
@@ -2324,6 +3341,21 @@
           <t>67f52a89981040986eab717d_product_defender_inspired_4x4</t>
         </is>
       </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>Karnataka Facility</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>Karnataka</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="1" t="n">
@@ -2349,6 +3381,21 @@
           <t>67f52a8a981040986eab7182_product_ev</t>
         </is>
       </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>Yixing Facility</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>Yixing</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="1" t="n">
@@ -2374,6 +3421,21 @@
           <t>67f52a8a981040986eab7182_product_electric_suv</t>
         </is>
       </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>Nanjing Facility</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>Nanjing</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="1" t="n">
@@ -2399,6 +3461,21 @@
           <t>67f52a8a981040986eab7182_product_sedan</t>
         </is>
       </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>Nanjing Facility</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>Nanjing</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="1" t="n">
@@ -2424,6 +3501,21 @@
           <t>67f52a8a981040986eab7182_product_mini_van</t>
         </is>
       </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>Nanjing Facility</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>Nanjing</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="1" t="n">
@@ -2449,6 +3541,21 @@
           <t>67f52a8a981040986eab7182_product_ev</t>
         </is>
       </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>Nevada Facility</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>Nevada</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="1" t="n">
@@ -2474,6 +3581,21 @@
           <t>67f52a8b981040986eab7186_product_tx5</t>
         </is>
       </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>Ansty Plant</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>Ansty</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="1" t="n">
@@ -2499,6 +3621,17 @@
           <t>67f52a8b981040986eab7186_product_eli</t>
         </is>
       </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>SFL Austria Plant</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr"/>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="1" t="n">
@@ -2524,6 +3657,17 @@
           <t>67f52a8c981040986eab7188_product_streetscooter</t>
         </is>
       </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>North Rhine-Westphalia</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr"/>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="1" t="n">
@@ -2549,6 +3693,21 @@
           <t>67f52a8d981040986eab718d_electric_buses</t>
         </is>
       </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>Hyderabad Facility</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>Hyderabad</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="1" t="n">
@@ -2574,6 +3733,21 @@
           <t>67f52a8f981040986eab7197_product_light_electric_vehicle_technology</t>
         </is>
       </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>Brisbane Facility</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>Brisbane</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="1" t="n">
@@ -2599,6 +3773,21 @@
           <t>67f52a94981040986eab71a8_product_tx_cab</t>
         </is>
       </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>Coventry Factory</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>Coventry</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="1" t="n">
@@ -2624,6 +3813,21 @@
           <t>67f52a95981040986eab71ab_electric_heavy_duty vehicles</t>
         </is>
       </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>Lancaster Plant</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>Lancaster</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="1" t="n">
@@ -2649,6 +3853,21 @@
           <t>67f52a96981040986eab71af_product_battery</t>
         </is>
       </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>Darwin Mini Gigafactory</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>Darwin</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="1" t="n">
@@ -2674,6 +3893,21 @@
           <t>67f52a96981040986eab71b0_product_ev_charging_tech</t>
         </is>
       </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>Port Elizabeth Plant</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>Port Elizabeth</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="1" t="n">
@@ -2699,6 +3933,21 @@
           <t>67f52a96981040986eab71b1_product_electric_suv</t>
         </is>
       </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>Shiyan Factory</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>Shiyan</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="1" t="n">
@@ -2724,6 +3973,21 @@
           <t>67f52a97981040986eab71b6_product_cathode_materials</t>
         </is>
       </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>Guizhou Guian New District Factory</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>Guizhou Guian New District</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="1" t="n">
@@ -2749,6 +4013,21 @@
           <t>67f52a99981040986eab71bc_product_ev_batteries</t>
         </is>
       </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>Townsville Battery Plant</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>Townsville</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="1" t="n">
@@ -2774,6 +4053,21 @@
           <t>67f52a99981040986eab71bc_product_home_battery_units</t>
         </is>
       </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>Townsville Battery Plant</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>Townsville</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="1" t="n">
@@ -2799,6 +4093,21 @@
           <t>67f52a99981040986eab71bd_product_electric_buses</t>
         </is>
       </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>Lancaster Facility</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>Lancaster</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="1" t="n">
@@ -2824,6 +4133,21 @@
           <t>67f52a9a981040986eab71c0_product_car_batteries</t>
         </is>
       </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>battery plant</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>Townsville</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="1" t="n">
@@ -2849,6 +4173,21 @@
           <t>67f52a9a981040986eab71c0_product_home_storage_units</t>
         </is>
       </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>battery plant</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>Townsville</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="1" t="n">
@@ -2874,6 +4213,21 @@
           <t>67f52a9a981040986eab71c0_product_microgrids</t>
         </is>
       </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>battery plant</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>Townsville</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="1" t="n">
@@ -2899,6 +4253,21 @@
           <t>67f52a9a981040986eab71c0_product_car_batteries</t>
         </is>
       </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>battery plant</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>IBM HQ Huron campus</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="1" t="n">
@@ -2924,6 +4293,21 @@
           <t>67f52a9a981040986eab71c0_product_home_storage_units</t>
         </is>
       </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>battery plant</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>IBM HQ Huron campus</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="1" t="n">
@@ -2949,6 +4333,21 @@
           <t>67f52a9a981040986eab71c0_product_microgrids</t>
         </is>
       </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>battery plant</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>IBM HQ Huron campus</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="1" t="n">
@@ -2974,6 +4373,21 @@
           <t>67f52a9b981040986eab71c3_product_electrode_paste</t>
         </is>
       </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>Suzhou Plant</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>Suzhou</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="1" t="n">
@@ -2999,6 +4413,21 @@
           <t>67f52a9b981040986eab71c3_product_electrode_paste</t>
         </is>
       </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>Suzhou Plant</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>Suzhou</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="1" t="n">
@@ -3024,6 +4453,21 @@
           <t>67f52a9c981040986eab71c7_product_li_ion_battery_systems</t>
         </is>
       </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>Darmstadt Facility</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>Darmstadt</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="1" t="n">
@@ -3049,6 +4493,21 @@
           <t>67f52a9c981040986eab71c7_product_li_ion_battery_systems</t>
         </is>
       </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>Darmstadt Facility</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>Darmstadt</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="1" t="n">
@@ -3074,6 +4533,17 @@
           <t>67f52a9d981040986eab71cd_product_battery_cells</t>
         </is>
       </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>German Gigafactory</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr"/>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="1" t="n">
@@ -3099,6 +4569,21 @@
           <t>67f52aa0981040986eab71d8_product_battery_cells</t>
         </is>
       </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>Liyang Gigafactory</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>Liyang</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="1" t="n">
@@ -3124,6 +4609,21 @@
           <t>67f52aa0981040986eab71d8_product_battery_cells</t>
         </is>
       </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>Liyang Gigafactory</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>Liyang</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="1" t="n">
@@ -3149,6 +4649,17 @@
           <t>67f52aa0981040986eab71d9_product_lithium_ion_battery</t>
         </is>
       </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>Northvolt Gigafactory</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr"/>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>Sweden</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="1" t="n">
@@ -3174,6 +4685,13 @@
           <t>67f52aa0981040986eab71da_product_zacua</t>
         </is>
       </c>
+      <c r="F110" t="inlineStr"/>
+      <c r="G110" t="inlineStr"/>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="1" t="n">
@@ -3199,6 +4717,13 @@
           <t>67f52aa0981040986eab71da_product_zacua</t>
         </is>
       </c>
+      <c r="F111" t="inlineStr"/>
+      <c r="G111" t="inlineStr"/>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="1" t="n">
@@ -3224,6 +4749,21 @@
           <t>67f52aa2981040986eab71df_product_tx_ecity</t>
         </is>
       </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>Coventry</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>Coventry</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="1" t="n">
@@ -3249,6 +4789,21 @@
           <t>67f52aa3981040986eab71e4_product_battery_electric_buses</t>
         </is>
       </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>California Plant</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>Los Angeles area</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="1" t="n">
@@ -3274,6 +4829,21 @@
           <t>67f52aa4981040986eab71e7_product_arrow_stf</t>
         </is>
       </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>Surendranagar Factory</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>Surendranagar</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="1" t="n">
@@ -3299,6 +4869,21 @@
           <t>67f52aa4981040986eab71e8_product_compact_sedans</t>
         </is>
       </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>Beijing EV Plant</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>Beijing</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="1" t="n">
@@ -3324,6 +4909,21 @@
           <t>67f52aa4981040986eab71e8_product_compact_crossover</t>
         </is>
       </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>Beijing EV Plant</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>Beijing</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="1" t="n">
@@ -3349,6 +4949,21 @@
           <t>67f52aa4981040986eab71e9_product_small_electric_suv</t>
         </is>
       </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>Shiyan Factory</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>Shiyan</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="1" t="n">
@@ -3374,6 +4989,21 @@
           <t>67f52aa5981040986eab71ed_product_youxia_x</t>
         </is>
       </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>Huzhou Factory</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>Huzhou</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="1" t="n">
@@ -3399,6 +5029,21 @@
           <t>67f52aa6981040986eab71f1_product_small_electric_suv</t>
         </is>
       </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>Dongfeng factory</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>Shiyan</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="1" t="n">
@@ -3424,6 +5069,21 @@
           <t>67f52aa7981040986eab71f3_product_electric_cars</t>
         </is>
       </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>Qinhuangdao Production Base</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>Qinhuangdao</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="1" t="n">
@@ -3449,6 +5109,21 @@
           <t>67f52aa7981040986eab71f3_product_new_energy_vehicles</t>
         </is>
       </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>Qinhuangdao Production Base</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>Qinhuangdao</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="1" t="n">
@@ -3474,6 +5149,21 @@
           <t>67f52aa7981040986eab71f4_product_aiways_rg</t>
         </is>
       </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>Shangrao Factory</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>Shangrao</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="1" t="n">
@@ -3499,6 +5189,21 @@
           <t>67f52aa7981040986eab71f6_product_battery_cells</t>
         </is>
       </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>Skellefteå Gigafactory</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>Skellefteå</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>Sweden</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="1" t="n">
@@ -3524,6 +5229,21 @@
           <t>67f52aa7981040986eab71f6_product_battery_cells</t>
         </is>
       </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>Skellefteå Gigafactory</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>Skellefteå</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>Sweden</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="1" t="n">
@@ -3549,6 +5269,21 @@
           <t>67f52aa8981040986eab71f7_product_electric_motors</t>
         </is>
       </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>Xiangyang Factory</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>Xiangyang</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="1" t="n">
@@ -3574,6 +5309,21 @@
           <t>67f52aa8981040986eab71f7_product_batteries</t>
         </is>
       </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>Xiangyang Factory</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>Xiangyang</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="1" t="n">
@@ -3599,6 +5349,13 @@
           <t>67f52aa9981040986eab71fd_product_nev</t>
         </is>
       </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>GAC NEV Plant</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr"/>
+      <c r="H127" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>